<commit_message>
Verify Publisher-rescue kit and link it from its niche
Re-ran the archive conversion on a copy: 9 of 10 sample files
converted with previews, index and contact sheet; the deliberately
damaged .pub fails with a clear reason.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DspfyLwNfeJ4CHdyACeRHQ
</commit_message>
<xml_diff>
--- a/kits/publisher-rescue/samples/st-aidans-wrenford/archive/index.xlsx
+++ b/kits/publisher-rescue/samples/st-aidans-wrenford/archive/index.xlsx
@@ -12,6 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Index'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,10 +33,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001E6B35"/>
     </font>
@@ -47,14 +50,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="009C1C1C"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
     </font>
   </fonts>
@@ -486,7 +492,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1128,6 +1134,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1171,7 +1178,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>07 October 2026, 10:36</t>
+          <t>07 October 2026, 10:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish and verify the kit fixes from the double-check
Each kit's fixes were re-tested by an independent verifier (all passed):
- cra-readiness: make_sbom.py no longer crashes with a relative --out on
  Node projects; examples write to the ignored clients/ folder.
- model-retirement: --from-raw re-applies grades without calling the
  paid API again; template placeholders are caught before any call.
- doc-accessibility, publisher-rescue: build scripts honour --help
  instead of overwriting files; the report states the real crawl delay;
  the sample delivery note names the substituted font.
- redcap-xlsform, replication-package: correct minimum Python versions;
  relative --python paths work; client folders are git-ignored.
- All kits: prices marked as estimates, how to put your name on the
  sample, the kit's own Python in skill commands, and other polish.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DspfyLwNfeJ4CHdyACeRHQ
</commit_message>
<xml_diff>
--- a/kits/publisher-rescue/samples/st-aidans-wrenford/archive/index.xlsx
+++ b/kits/publisher-rescue/samples/st-aidans-wrenford/archive/index.xlsx
@@ -629,7 +629,11 @@
           <t>LiberationSans-Bold, LiberationSerif, Z003-MediumItalic</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Some text is shown in a stand-in font (Z003-MediumItalic) because the font the file asked for was not available, so it can look different from the original.</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="n">
         <v>50.7</v>
       </c>
@@ -1178,7 +1182,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>07 October 2026, 10:37</t>
+          <t>07 October 2026, 15:19</t>
         </is>
       </c>
     </row>

</xml_diff>